<commit_message>
Corrida | ARG-IGA | 2026-06-17 12:00:14.749737
</commit_message>
<xml_diff>
--- a/indicadores/ARG-IGA_out.xlsx
+++ b/indicadores/ARG-IGA_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="548">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="550">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">td1coef</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Argentina</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">01/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2160,9 +2166,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2173,7 +2183,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2187,7 +2197,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -2203,7 +2213,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2231,7 +2241,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2245,7 +2255,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -2273,7 +2283,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2287,7 +2297,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2301,7 +2311,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2315,7 +2325,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -2331,7 +2341,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2345,7 +2355,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -2493,10 +2503,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2509,10 +2519,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2536,66 +2546,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>89.1603664077652</v>
@@ -2648,7 +2658,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>77.6519088211317</v>
@@ -2705,7 +2715,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>92.0576555753691</v>
@@ -2762,7 +2772,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>94.2709747263278</v>
@@ -2819,7 +2829,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>94.3323342950231</v>
@@ -2876,7 +2886,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>95.981546938396</v>
@@ -2933,7 +2943,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>97.6508920935309</v>
@@ -2990,7 +3000,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>95.6394488141339</v>
@@ -3047,7 +3057,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>96.8925542466303</v>
@@ -3104,7 +3114,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>97.0956107678397</v>
@@ -3161,7 +3171,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>98.2666834156512</v>
@@ -3218,7 +3228,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>99.0049640034812</v>
@@ -3275,7 +3285,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>96.4372963527475</v>
@@ -3334,7 +3344,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>85.8420130490678</v>
@@ -3393,7 +3403,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>98.6649192201423</v>
@@ -3452,7 +3462,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>102.469084212175</v>
@@ -3511,7 +3521,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>103.034329314501</v>
@@ -3570,7 +3580,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>99.9125722149562</v>
@@ -3629,7 +3639,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>101.402282236919</v>
@@ -3688,7 +3698,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>102.246103937838</v>
@@ -3747,7 +3757,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>102.868159236805</v>
@@ -3806,7 +3816,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>101.634978715338</v>
@@ -3865,7 +3875,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>103.089545082429</v>
@@ -3924,7 +3934,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>102.398716427081</v>
@@ -3983,7 +3993,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>94.9484401673342</v>
@@ -4042,7 +4052,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>93.0262813575362</v>
@@ -4101,7 +4111,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>99.9582549251639</v>
@@ -4160,7 +4170,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>97.4039323754577</v>
@@ -4219,7 +4229,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>103.165149723691</v>
@@ -4278,7 +4288,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>95.71317231569</v>
@@ -4337,7 +4347,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>98.0212716368035</v>
@@ -4396,7 +4406,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>96.158237664898</v>
@@ -4455,7 +4465,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>94.5854497565786</v>
@@ -4514,7 +4524,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>96.4201405947286</v>
@@ -4573,7 +4583,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>96.3907424444961</v>
@@ -4632,7 +4642,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>94.9180754081156</v>
@@ -4691,7 +4701,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>91.2899048739815</v>
@@ -4750,7 +4760,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>90.0622313402955</v>
@@ -4809,7 +4819,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>99.2880999148388</v>
@@ -4868,7 +4878,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>101.026876444466</v>
@@ -4927,7 +4937,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>103.722080075107</v>
@@ -4986,7 +4996,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>101.236884575935</v>
@@ -5045,7 +5055,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>106.322895858665</v>
@@ -5104,7 +5114,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>103.494440302704</v>
@@ -5163,7 +5173,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>101.105088646272</v>
@@ -5222,7 +5232,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>106.610248643364</v>
@@ -5281,7 +5291,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>103.948942429223</v>
@@ -5340,7 +5350,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>102.919629856395</v>
@@ -5399,7 +5409,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>101.047578074132</v>
@@ -5458,7 +5468,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>96.8700403795247</v>
@@ -5517,7 +5527,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>105.203832039407</v>
@@ -5576,7 +5586,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>110.889853505701</v>
@@ -5635,7 +5645,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>110.919677087856</v>
@@ -5694,7 +5704,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>108.32106561868</v>
@@ -5753,7 +5763,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>114.556986537314</v>
@@ -5812,7 +5822,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>110.629064899507</v>
@@ -5871,7 +5881,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>113.82699186941</v>
@@ -5930,7 +5940,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>117.782154857424</v>
@@ -5989,7 +5999,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>111.302421154787</v>
@@ -6048,7 +6058,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>110.034464518657</v>
@@ -6107,7 +6117,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>105.53876109402</v>
@@ -6166,7 +6176,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>102.35638034549</v>
@@ -6225,7 +6235,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>114.787509522638</v>
@@ -6284,7 +6294,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>117.379169981127</v>
@@ -6343,7 +6353,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>118.267718127633</v>
@@ -6402,7 +6412,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>119.989265458143</v>
@@ -6461,7 +6471,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>118.875427690828</v>
@@ -6520,7 +6530,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>115.745287265669</v>
@@ -6579,7 +6589,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>116.207634258772</v>
@@ -6638,7 +6648,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>114.805132556893</v>
@@ -6697,7 +6707,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>112.49015583757</v>
@@ -6756,7 +6766,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>107.787150465259</v>
@@ -6815,7 +6825,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>103.82304958337</v>
@@ -6874,7 +6884,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>99.1207046409332</v>
@@ -6933,7 +6943,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>110.223752540625</v>
@@ -6992,7 +7002,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>111.516373184305</v>
@@ -7051,7 +7061,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>112.070430536469</v>
@@ -7110,7 +7120,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>112.577028765088</v>
@@ -7169,7 +7179,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>111.278335218954</v>
@@ -7228,7 +7238,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>111.166425646458</v>
@@ -7287,7 +7297,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>111.46035987421</v>
@@ -7346,7 +7356,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>111.689523988872</v>
@@ -7405,7 +7415,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>113.264716053586</v>
@@ -7464,7 +7474,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>112.036575111948</v>
@@ -7523,7 +7533,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>104.937947084129</v>
@@ -7582,7 +7592,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>100.665834253884</v>
@@ -7641,7 +7651,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>110.471842253355</v>
@@ -7700,7 +7710,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>110.09406820891</v>
@@ -7759,7 +7769,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>112.875464702925</v>
@@ -7818,7 +7828,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>111.219063192363</v>
@@ -7877,7 +7887,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>110.761288846009</v>
@@ -7936,7 +7946,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>112.147049822026</v>
@@ -7995,7 +8005,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>109.648306317385</v>
@@ -8054,7 +8064,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>109.655097605887</v>
@@ -8113,7 +8123,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>110.244623888822</v>
@@ -8172,7 +8182,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>109.662823203896</v>
@@ -8231,7 +8241,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>104.144272785142</v>
@@ -8290,7 +8300,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>97.4388946342783</v>
@@ -8349,7 +8359,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>105.757610641593</v>
@@ -8408,7 +8418,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>110.782207699111</v>
@@ -8467,7 +8477,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>113.142893160692</v>
@@ -8526,7 +8536,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>110.463890446388</v>
@@ -8585,7 +8595,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>108.019573551823</v>
@@ -8644,7 +8654,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>105.706161592434</v>
@@ -8703,7 +8713,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>99.8183158072613</v>
@@ -8762,7 +8772,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>100.829767844484</v>
@@ -8821,7 +8831,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>99.7107622789141</v>
@@ -8880,7 +8890,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>91.1435096821605</v>
@@ -8939,7 +8949,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>88.5574762813517</v>
@@ -8998,7 +9008,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>84.2504871060022</v>
@@ -9057,7 +9067,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>89.2113012011094</v>
@@ -9116,7 +9126,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>97.8743403245512</v>
@@ -9175,7 +9185,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>100.908669912545</v>
@@ -9234,7 +9244,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>97.3920514448711</v>
@@ -9293,7 +9303,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>95.5625498201471</v>
@@ -9352,7 +9362,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>93.3184914370506</v>
@@ -9411,7 +9421,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>91.5684913896386</v>
@@ -9470,7 +9480,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>94.2029006445221</v>
@@ -9529,7 +9539,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>93.1529739701749</v>
@@ -9588,7 +9598,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>91.5422084468385</v>
@@ -9647,7 +9657,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>93.2132949567945</v>
@@ -9706,7 +9716,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>88.6538307625632</v>
@@ -9765,7 +9775,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>95.7638563868669</v>
@@ -9824,7 +9834,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>104.197637291049</v>
@@ -9883,7 +9893,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>107.54261789406</v>
@@ -9942,7 +9952,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>105.183727002447</v>
@@ -10001,7 +10011,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>103.993402881461</v>
@@ -10060,7 +10070,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>101.210659866138</v>
@@ -10119,7 +10129,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>102.087886911386</v>
@@ -10178,7 +10188,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>105.15861740252</v>
@@ -10237,7 +10247,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>103.169865708848</v>
@@ -10296,7 +10306,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>102.242345229383</v>
@@ -10355,7 +10365,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>103.228296382425</v>
@@ -10414,7 +10424,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>98.3987759349017</v>
@@ -10473,7 +10483,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>108.432824367185</v>
@@ -10532,7 +10542,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>109.619645572055</v>
@@ -10591,7 +10601,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>114.294032242369</v>
@@ -10650,7 +10660,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>113.66035775534</v>
@@ -10709,7 +10719,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>111.934077181318</v>
@@ -10768,7 +10778,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>111.193297978599</v>
@@ -10827,7 +10837,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>111.265602315713</v>
@@ -10886,7 +10896,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>112.005691897197</v>
@@ -10945,7 +10955,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>113.117570026842</v>
@@ -11004,7 +11014,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>111.60826335603</v>
@@ -11063,7 +11073,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>110.950185975985</v>
@@ -11122,7 +11132,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>104.584169314459</v>
@@ -11181,7 +11191,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>115.360144431936</v>
@@ -11240,7 +11250,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>121.269877780511</v>
@@ -11299,7 +11309,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>126.753891746558</v>
@@ -11358,7 +11368,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>124.770633661761</v>
@@ -11417,7 +11427,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>120.117087165548</v>
@@ -11476,7 +11486,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>121.487773347679</v>
@@ -11535,7 +11545,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>120.815726069876</v>
@@ -11594,7 +11604,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>120.663652288193</v>
@@ -11653,7 +11663,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>122.941637381587</v>
@@ -11712,7 +11722,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>120.902905795501</v>
@@ -11771,7 +11781,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>118.835063487993</v>
@@ -11830,7 +11840,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>114.50363840737</v>
@@ -11889,7 +11899,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>126.193943226409</v>
@@ -11948,7 +11958,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>128.993170801529</v>
@@ -12007,7 +12017,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>135.43589065866</v>
@@ -12066,7 +12076,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>133.999764551246</v>
@@ -12125,7 +12135,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>131.50248102841</v>
@@ -12184,7 +12194,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>132.137590018531</v>
@@ -12243,7 +12253,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>131.281275614541</v>
@@ -12302,7 +12312,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>132.091206990211</v>
@@ -12361,7 +12371,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>134.352546097549</v>
@@ -12420,7 +12430,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>130.624733694558</v>
@@ -12479,7 +12489,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>127.177159980779</v>
@@ -12538,7 +12548,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>122.778507130415</v>
@@ -12597,7 +12607,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>135.603634238998</v>
@@ -12656,7 +12666,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>140.913867540139</v>
@@ -12715,7 +12725,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>147.802161893212</v>
@@ -12774,7 +12784,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>144.999765452776</v>
@@ -12833,7 +12843,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>140.346271644501</v>
@@ -12892,7 +12902,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>143.851806487379</v>
@@ -12951,7 +12961,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>142.461158543753</v>
@@ -13010,7 +13020,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>145.757436057785</v>
@@ -13069,7 +13079,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>147.203058763452</v>
@@ -13128,7 +13138,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>142.612503740254</v>
@@ -13187,7 +13197,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>139.723751689443</v>
@@ -13246,7 +13256,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>131.331177564101</v>
@@ -13305,7 +13315,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>136.099372674854</v>
@@ -13364,7 +13374,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>150.8070768115</v>
@@ -13423,7 +13433,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>154.025214349235</v>
@@ -13482,7 +13492,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>145.843130298949</v>
@@ -13541,7 +13551,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>151.369440712429</v>
@@ -13600,7 +13610,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>146.619296652799</v>
@@ -13659,7 +13669,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>150.955055371256</v>
@@ -13718,7 +13728,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>144.902579905037</v>
@@ -13777,7 +13787,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>138.298252206445</v>
@@ -13836,7 +13846,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>134.657935737381</v>
@@ -13895,7 +13905,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>130.379945335183</v>
@@ -13954,7 +13964,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>122.22090764407</v>
@@ -14013,7 +14023,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>134.086934936288</v>
@@ -14072,7 +14082,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>139.811791904581</v>
@@ -14131,7 +14141,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>141.485031370722</v>
@@ -14190,7 +14200,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>141.555446308688</v>
@@ -14249,7 +14259,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>144.255655604331</v>
@@ -14308,7 +14318,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>141.628560896932</v>
@@ -14367,7 +14377,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>142.706675180979</v>
@@ -14426,7 +14436,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>140.782825975869</v>
@@ -14485,7 +14495,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>139.625348252876</v>
@@ -14544,7 +14554,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>137.112693030757</v>
@@ -14603,7 +14613,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>134.353511123674</v>
@@ -14662,7 +14672,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>128.739910725709</v>
@@ -14721,7 +14731,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>143.733272665084</v>
@@ -14780,7 +14790,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>154.277916187926</v>
@@ -14839,7 +14849,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>155.584427544439</v>
@@ -14898,7 +14908,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>156.009391409799</v>
@@ -14957,7 +14967,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>153.515772485281</v>
@@ -15016,7 +15026,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>155.084580565063</v>
@@ -15075,7 +15085,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>155.255922088068</v>
@@ -15134,7 +15144,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>149.866197148099</v>
@@ -15193,7 +15203,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>153.093998720061</v>
@@ -15252,7 +15262,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>149.112438712529</v>
@@ -15311,7 +15321,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>145.309722477115</v>
@@ -15370,7 +15380,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>136.493426281942</v>
@@ -15429,7 +15439,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>153.202594674293</v>
@@ -15488,7 +15498,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>159.220509030752</v>
@@ -15547,7 +15557,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>164.472857223666</v>
@@ -15606,7 +15616,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>162.833759731612</v>
@@ -15665,7 +15675,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>161.499415776895</v>
@@ -15724,7 +15734,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>162.65893262969</v>
@@ -15783,7 +15793,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>164.086996473228</v>
@@ -15842,7 +15852,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>157.212159358099</v>
@@ -15901,7 +15911,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>157.641892661487</v>
@@ -15960,7 +15970,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>152.221430812244</v>
@@ -16019,7 +16029,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>148.810936083815</v>
@@ -16078,7 +16088,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>141.892543960568</v>
@@ -16137,7 +16147,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>159.039102018204</v>
@@ -16196,7 +16206,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>144.902827488279</v>
@@ -16255,7 +16265,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>161.189199749428</v>
@@ -16314,7 +16324,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>145.547606469385</v>
@@ -16373,7 +16383,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>161.32677051482</v>
@@ -16432,7 +16442,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>161.602530619242</v>
@@ -16491,7 +16501,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>159.033149859159</v>
@@ -16550,7 +16560,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>158.679579206969</v>
@@ -16609,7 +16619,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>155.877254962925</v>
@@ -16668,7 +16678,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>151.794429163537</v>
@@ -16727,7 +16737,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>149.57907851277</v>
@@ -16786,7 +16796,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>141.818800985007</v>
@@ -16845,7 +16855,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>159.692862442152</v>
@@ -16904,7 +16914,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>167.45547368541</v>
@@ -16963,7 +16973,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>173.087240298255</v>
@@ -17022,7 +17032,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>164.293385076371</v>
@@ -17081,7 +17091,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>167.742843693103</v>
@@ -17140,7 +17150,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>167.817774956811</v>
@@ -17199,7 +17209,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>166.746461867423</v>
@@ -17258,7 +17268,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>164.987830473175</v>
@@ -17317,7 +17327,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>159.219742820668</v>
@@ -17376,7 +17386,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>154.199996389618</v>
@@ -17435,7 +17445,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>152.986248572176</v>
@@ -17494,7 +17504,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>144.451911374426</v>
@@ -17553,7 +17563,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>154.108512587612</v>
@@ -17612,7 +17622,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>164.266679027071</v>
@@ -17671,7 +17681,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>168.333697765545</v>
@@ -17730,7 +17740,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>163.498576296853</v>
@@ -17789,7 +17799,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>161.072853085137</v>
@@ -17848,7 +17858,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>157.637236048974</v>
@@ -17907,7 +17917,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>160.625268647459</v>
@@ -17966,7 +17976,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>157.935254411551</v>
@@ -18025,7 +18035,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>152.362732070472</v>
@@ -18084,7 +18094,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>148.484245494626</v>
@@ -18143,7 +18153,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>149.109877194424</v>
@@ -18202,7 +18212,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>141.75317929432</v>
@@ -18261,7 +18271,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>156.487447231013</v>
@@ -18320,7 +18330,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>168.806906978296</v>
@@ -18379,7 +18389,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>168.154039783161</v>
@@ -18438,7 +18448,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>171.708831992263</v>
@@ -18497,7 +18507,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>167.797629380852</v>
@@ -18556,7 +18566,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>164.118804602942</v>
@@ -18615,7 +18625,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>164.593827620958</v>
@@ -18674,7 +18684,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>161.716995197807</v>
@@ -18733,7 +18743,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>156.05965021135</v>
@@ -18792,7 +18802,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>152.024043629191</v>
@@ -18851,7 +18861,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>152.414699654277</v>
@@ -18910,7 +18920,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>145.430893633987</v>
@@ -18969,7 +18979,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>157.230687581589</v>
@@ -19028,7 +19038,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>162.921273184389</v>
@@ -19087,7 +19097,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>166.08508314835</v>
@@ -19146,7 +19156,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>162.722451017368</v>
@@ -19205,7 +19215,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>157.463706602704</v>
@@ -19264,7 +19274,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>159.427653920969</v>
@@ -19323,7 +19333,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>157.048280407651</v>
@@ -19382,7 +19392,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>154.592593958041</v>
@@ -19441,7 +19451,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>154.612356301712</v>
@@ -19500,7 +19510,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>151.988961470897</v>
@@ -19559,7 +19569,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>153.564905769606</v>
@@ -19618,7 +19628,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>141.801731697051</v>
@@ -19677,7 +19687,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>162.04047499423</v>
@@ -19736,7 +19746,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>164.920214173236</v>
@@ -19795,7 +19805,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>172.76007352517</v>
@@ -19854,7 +19864,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>170.047649373423</v>
@@ -19913,7 +19923,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>167.947567975244</v>
@@ -19972,7 +19982,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>170.32527506664</v>
@@ -20031,7 +20041,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>166.687175331258</v>
@@ -20090,7 +20100,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>166.382613087523</v>
@@ -20149,7 +20159,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>165.159316629873</v>
@@ -20208,7 +20218,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>157.672994372982</v>
@@ -20267,7 +20277,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>159.41702030653</v>
@@ -20326,7 +20336,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>150.124060226126</v>
@@ -20385,7 +20395,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>166.023136585157</v>
@@ -20444,7 +20454,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>163.557942692441</v>
@@ -20503,7 +20513,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>167.56168514234</v>
@@ -20562,7 +20572,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>161.17282343045</v>
@@ -20621,7 +20631,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>163.867706344336</v>
@@ -20680,7 +20690,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>165.794480805171</v>
@@ -20739,7 +20749,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>157.483429776097</v>
@@ -20798,7 +20808,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>157.577189285828</v>
@@ -20857,7 +20867,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>152.851195323542</v>
@@ -20916,7 +20926,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>146.452641390336</v>
@@ -20975,7 +20985,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>148.990652505572</v>
@@ -21034,7 +21044,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>141.376619159862</v>
@@ -21093,7 +21103,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>152.374667325888</v>
@@ -21152,7 +21162,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>160.928704788353</v>
@@ -21211,7 +21221,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>167.696734428985</v>
@@ -21270,7 +21280,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>162.808713021862</v>
@@ -21329,7 +21339,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>160.364702318301</v>
@@ -21388,7 +21398,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>158.672694908143</v>
@@ -21447,7 +21457,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>153.690673089344</v>
@@ -21506,7 +21516,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>155.100679264476</v>
@@ -21565,7 +21575,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>149.742655798976</v>
@@ -21624,7 +21634,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>142.786625334993</v>
@@ -21683,7 +21693,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>143.444628216721</v>
@@ -21742,7 +21752,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>136.394597341063</v>
@@ -21801,7 +21811,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>137.71060310452</v>
@@ -21860,7 +21870,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>125.020547528335</v>
@@ -21919,7 +21929,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>136.770598987765</v>
@@ -21978,7 +21988,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>145.042635215204</v>
@@ -22037,7 +22047,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>142.03462204159</v>
@@ -22096,7 +22106,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>143.444628216721</v>
@@ -22155,7 +22165,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>145.606637685257</v>
@@ -22214,7 +22224,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>148.144648800493</v>
@@ -22273,7 +22283,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>151.434663209134</v>
@@ -22332,7 +22342,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>142.786625334993</v>
@@ -22391,7 +22401,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>146.076639743634</v>
@@ -22450,7 +22460,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>137.522602281169</v>
@@ -22509,7 +22519,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>154.160675147722</v>
@@ -22568,7 +22578,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>157.07468790966</v>
@@ -22627,7 +22637,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>154.724677617774</v>
@@ -22686,7 +22696,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>158.296693261441</v>
@@ -22745,7 +22755,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>151.152661974108</v>
@@ -22804,7 +22814,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>154.348675971072</v>
@@ -22863,7 +22873,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>157.262688733011</v>
@@ -22922,7 +22932,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>157.732690791388</v>
@@ -22981,7 +22991,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>160.364702318301</v>
@@ -23040,7 +23050,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>159.048696554844</v>
@@ -23099,7 +23109,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>150.024657034002</v>
@@ -23158,7 +23168,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>147.956647977143</v>
@@ -23217,7 +23227,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>159.800699848248</v>
@@ -23276,7 +23286,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>164.406720020345</v>
@@ -23335,7 +23345,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>166.380728665529</v>
@@ -23394,7 +23404,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>168.82473936909</v>
@@ -23453,7 +23463,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>160.928704788353</v>
@@ -23512,7 +23522,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>165.158723313748</v>
@@ -23571,7 +23581,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>163.184714668564</v>
@@ -23630,7 +23640,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>160.364702318301</v>
@@ -23689,7 +23699,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>164.124718785318</v>
@@ -23748,7 +23758,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>159.14269696652</v>
@@ -23807,7 +23817,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>151.71666444416</v>
@@ -23866,7 +23876,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>147.298645095414</v>
@@ -23925,7 +23935,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>160.646703553327</v>
@@ -23984,7 +23994,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>158.390693673116</v>
@@ -24043,7 +24053,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>159.706699436573</v>
@@ -24102,7 +24112,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>159.800699848248</v>
@@ -24161,7 +24171,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>159.800699848248</v>
@@ -24220,7 +24230,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>164.50072043202</v>
@@ -24279,7 +24289,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>162.714712610187</v>
@@ -24338,7 +24348,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>161.022705200029</v>
@@ -24397,7 +24407,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>161.116705611704</v>
@@ -24456,7 +24466,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>150.212657857353</v>
@@ -24515,7 +24525,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>143.350627805046</v>
@@ -24574,7 +24584,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>139.590611338028</v>
@@ -24633,7 +24643,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>142.974626158344</v>
@@ -24692,7 +24702,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>155.758682146204</v>
@@ -24751,7 +24761,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>156.416685027932</v>
@@ -24810,7 +24820,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B379" s="2" t="n">
         <v>154.254675559397</v>
@@ -24869,7 +24879,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B380" s="2" t="n">
         <v>156.416685027932</v>
@@ -24928,7 +24938,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B381" s="2" t="n">
         <v>156.604685851283</v>
@@ -24987,7 +24997,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B382" s="2" t="n">
         <v>157.732690791388</v>
@@ -25046,7 +25056,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B383" s="2" t="n">
         <v>163.090714256888</v>
@@ -25105,7 +25115,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B384" s="2" t="n">
         <v>161.680708081757</v>
@@ -25164,7 +25174,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B385" s="2" t="n">
         <v>156.416685027932</v>
@@ -25223,7 +25233,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B386" s="2" t="n">
         <v>153.596672677669</v>
@@ -25282,7 +25292,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B387" s="2" t="n">
         <v>149.6486553873</v>
@@ -25341,7 +25351,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B388" s="2" t="n">
         <v>153.314671442643</v>
@@ -25400,7 +25410,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B389" s="2" t="n">
         <v>164.782721667046</v>
@@ -25459,7 +25469,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B390" s="2" t="n">
         <v>164.312719608669</v>
@@ -25518,7 +25528,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B391" s="2" t="n">
         <v>165.722725783801</v>
@@ -25577,7 +25587,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B392" s="2" t="n">
         <v>160.928704788353</v>
@@ -25636,7 +25646,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B393" s="2" t="n">
         <v>163.46671590359</v>
@@ -25695,7 +25705,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B394" s="2" t="n">
         <v>166.662729900555</v>
@@ -25754,7 +25764,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B395" s="2" t="n">
         <v>168.918739780766</v>
@@ -25813,7 +25823,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B396" s="2" t="n">
         <v>162.338710963485</v>
@@ -25872,7 +25882,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B397" s="2" t="n">
         <v>159.048696554844</v>
@@ -25931,7 +25941,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B398" s="2" t="n">
         <v>151.998665679186</v>
@@ -25990,7 +26000,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B399" s="2" t="n">
         <v>144.760633980178</v>
@@ -26049,7 +26059,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B400" s="2" t="n">
         <v>158.014692026415</v>
@@ -26108,7 +26118,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B401" s="2" t="n">
         <v>164.782721667046</v>
@@ -26167,7 +26177,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B402" s="2"/>
       <c r="C402" s="3" t="n">
@@ -26200,7 +26210,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B403" s="2"/>
       <c r="C403" s="3" t="n">
@@ -26233,7 +26243,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B404" s="2"/>
       <c r="C404" s="3" t="n">
@@ -26266,7 +26276,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B405" s="2"/>
       <c r="C405" s="3" t="n">
@@ -26299,7 +26309,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B406" s="2"/>
       <c r="C406" s="3" t="n">
@@ -26332,7 +26342,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B407" s="2"/>
       <c r="C407" s="3" t="n">
@@ -26365,7 +26375,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B408" s="2"/>
       <c r="C408" s="3" t="n">
@@ -26398,7 +26408,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B409" s="2"/>
       <c r="C409" s="3" t="n">
@@ -26431,7 +26441,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B410" s="2"/>
       <c r="C410" s="3" t="n">
@@ -26464,7 +26474,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B411" s="2"/>
       <c r="C411" s="3" t="n">
@@ -26497,7 +26507,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B412" s="2"/>
       <c r="C412" s="3" t="n">
@@ -26530,7 +26540,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B413" s="2"/>
       <c r="C413" s="3" t="n">
@@ -26563,7 +26573,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B414" s="2"/>
       <c r="C414" s="3"/>
@@ -26586,7 +26596,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B415" s="2"/>
       <c r="C415" s="3"/>
@@ -26609,7 +26619,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3"/>
@@ -26632,7 +26642,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3"/>
@@ -26655,7 +26665,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3"/>
@@ -26678,7 +26688,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3"/>
@@ -26701,7 +26711,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3"/>
@@ -26724,7 +26734,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3"/>
@@ -26747,7 +26757,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B422" s="2"/>
       <c r="C422" s="3"/>
@@ -26770,7 +26780,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B423" s="2"/>
       <c r="C423" s="3"/>
@@ -26793,7 +26803,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B424" s="2"/>
       <c r="C424" s="3"/>
@@ -26816,7 +26826,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B425" s="2"/>
       <c r="C425" s="3"/>
@@ -26839,7 +26849,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3"/>
@@ -26862,7 +26872,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3"/>
@@ -26885,7 +26895,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3"/>
@@ -26908,7 +26918,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3"/>
@@ -26931,7 +26941,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3"/>
@@ -26954,7 +26964,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3"/>
@@ -26977,7 +26987,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3"/>
@@ -27000,7 +27010,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3"/>
@@ -27023,7 +27033,7 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B434" s="2"/>
       <c r="C434" s="3"/>
@@ -27046,7 +27056,7 @@
     </row>
     <row r="435">
       <c r="A435" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B435" s="2"/>
       <c r="C435" s="3"/>
@@ -27069,7 +27079,7 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B436" s="2"/>
       <c r="C436" s="3"/>
@@ -27092,7 +27102,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B437" s="2"/>
       <c r="C437" s="3"/>
@@ -27115,7 +27125,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B438" s="2"/>
       <c r="C438" s="3"/>
@@ -27138,7 +27148,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B439" s="2"/>
       <c r="C439" s="3"/>
@@ -27161,7 +27171,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B440" s="2"/>
       <c r="C440" s="3"/>
@@ -27184,7 +27194,7 @@
     </row>
     <row r="441">
       <c r="A441" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B441" s="2"/>
       <c r="C441" s="3"/>
@@ -27207,7 +27217,7 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B442" s="2"/>
       <c r="C442" s="3"/>
@@ -27230,7 +27240,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B443" s="2"/>
       <c r="C443" s="3"/>
@@ -27253,7 +27263,7 @@
     </row>
     <row r="444">
       <c r="A444" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B444" s="2"/>
       <c r="C444" s="3"/>
@@ -27276,7 +27286,7 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B445" s="2"/>
       <c r="C445" s="3"/>
@@ -27299,7 +27309,7 @@
     </row>
     <row r="446">
       <c r="A446" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B446" s="2"/>
       <c r="C446" s="3"/>
@@ -27322,7 +27332,7 @@
     </row>
     <row r="447">
       <c r="A447" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B447" s="2"/>
       <c r="C447" s="3"/>
@@ -27345,7 +27355,7 @@
     </row>
     <row r="448">
       <c r="A448" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B448" s="2"/>
       <c r="C448" s="3"/>
@@ -27368,7 +27378,7 @@
     </row>
     <row r="449">
       <c r="A449" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B449" s="2"/>
       <c r="C449" s="3"/>
@@ -27391,7 +27401,7 @@
     </row>
     <row r="450">
       <c r="A450" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B450" s="2"/>
       <c r="C450" s="3"/>
@@ -27414,7 +27424,7 @@
     </row>
     <row r="451">
       <c r="A451" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B451" s="2"/>
       <c r="C451" s="3"/>
@@ -27437,7 +27447,7 @@
     </row>
     <row r="452">
       <c r="A452" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B452" s="2"/>
       <c r="C452" s="3"/>
@@ -27460,7 +27470,7 @@
     </row>
     <row r="453">
       <c r="A453" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B453" s="2"/>
       <c r="C453" s="3"/>
@@ -27483,7 +27493,7 @@
     </row>
     <row r="454">
       <c r="A454" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B454" s="2"/>
       <c r="C454" s="3"/>
@@ -27506,7 +27516,7 @@
     </row>
     <row r="455">
       <c r="A455" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B455" s="2"/>
       <c r="C455" s="3"/>
@@ -27529,7 +27539,7 @@
     </row>
     <row r="456">
       <c r="A456" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B456" s="2"/>
       <c r="C456" s="3"/>
@@ -27552,7 +27562,7 @@
     </row>
     <row r="457">
       <c r="A457" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B457" s="2"/>
       <c r="C457" s="3"/>
@@ -27586,97 +27596,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
   </sheetData>
@@ -27700,7 +27710,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -27710,13 +27720,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.110211378964954</v>
@@ -27724,7 +27734,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.189502422637383</v>
@@ -27732,7 +27742,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.254472960577932</v>
@@ -27740,7 +27750,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.322252001265812</v>
@@ -27748,7 +27758,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.396237940149816</v>
@@ -27756,7 +27766,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.455921877822756</v>
@@ -27764,7 +27774,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.512570706860491</v>
@@ -27772,7 +27782,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.589370928451048</v>
@@ -27780,7 +27790,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.654871784374016</v>
@@ -27788,7 +27798,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.661939040140289</v>
@@ -27796,7 +27806,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.610449202530784</v>
@@ -27804,7 +27814,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.518343876276005</v>
@@ -27812,7 +27822,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.430276178880569</v>
@@ -27820,7 +27830,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.359008795474511</v>
@@ -27828,7 +27838,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.272395239870305</v>
@@ -27836,7 +27846,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0.154517463216336</v>
@@ -27844,7 +27854,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>0.0602327521728908</v>
@@ -27852,7 +27862,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>0.0154169941219144</v>
@@ -27860,7 +27870,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>-0.0316951077216745</v>

</xml_diff>